<commit_message>
chore(data-release): publish site data 2026-09-11 17:11:19 UTC
</commit_message>
<xml_diff>
--- a/countries/ch/2026-2029.xlsx
+++ b/countries/ch/2026-2029.xlsx
@@ -20408,13 +20408,13 @@
         </is>
       </c>
       <c r="N135" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="O135" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="R135" t="n">
-        <v>1.232265643612346</v>
+        <v>1.243367135897142</v>
       </c>
       <c r="S135" t="inlineStr">
         <is>
@@ -25731,13 +25731,13 @@
         </is>
       </c>
       <c r="N171" t="n">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="O171" t="n">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="R171" t="n">
-        <v>1.476498473877856</v>
+        <v>1.532005935301835</v>
       </c>
       <c r="S171" t="inlineStr">
         <is>
@@ -30329,13 +30329,13 @@
         </is>
       </c>
       <c r="N202" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="O202" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="R202" t="n">
-        <v>1.820644734706529</v>
+        <v>1.831746226991325</v>
       </c>
       <c r="S202" t="inlineStr">
         <is>
@@ -30909,13 +30909,13 @@
         </is>
       </c>
       <c r="N206" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O206" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R206" t="n">
-        <v>0.07771044599357135</v>
+        <v>0.08881193827836725</v>
       </c>
       <c r="S206" t="inlineStr">
         <is>
@@ -31054,13 +31054,13 @@
         </is>
       </c>
       <c r="N207" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O207" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R207" t="n">
-        <v>0.06660895370877544</v>
+        <v>0.07771044599357135</v>
       </c>
       <c r="S207" t="inlineStr">
         <is>
@@ -31924,13 +31924,13 @@
         </is>
       </c>
       <c r="N213" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O213" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R213" t="n">
-        <v>0.2442328302655099</v>
+        <v>0.2553343225503059</v>
       </c>
       <c r="S213" t="inlineStr">
         <is>
@@ -32794,13 +32794,13 @@
         </is>
       </c>
       <c r="N219" t="n">
-        <v>243</v>
+        <v>267</v>
       </c>
       <c r="O219" t="n">
-        <v>243</v>
+        <v>267</v>
       </c>
       <c r="R219" t="n">
-        <v>2.697662625205405</v>
+        <v>2.964098440040507</v>
       </c>
       <c r="S219" t="inlineStr">
         <is>
@@ -33157,6 +33157,1166 @@
         </is>
       </c>
       <c r="BC221" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>D004</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>新型冠状病毒感染</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N222" t="n">
+        <v>113</v>
+      </c>
+      <c r="O222" t="n">
+        <v>113</v>
+      </c>
+      <c r="R222" t="n">
+        <v>1.254468628181937</v>
+      </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO222" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP222" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR222" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS222" t="inlineStr"/>
+      <c r="AT222" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU222" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV222" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW222" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX222" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY222" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ222" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA222" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB222" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC222" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>D007</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Hepatitis A</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>甲型肝炎</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N223" t="n">
+        <v>10</v>
+      </c>
+      <c r="O223" t="n">
+        <v>10</v>
+      </c>
+      <c r="R223" t="n">
+        <v>0.1110149228479591</v>
+      </c>
+      <c r="S223" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO223" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP223" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR223" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS223" t="inlineStr"/>
+      <c r="AT223" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU223" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV223" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW223" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX223" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY223" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ223" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA223" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB223" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC223" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>D011</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Hepatitis E</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>戊型肝炎</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N224" t="n">
+        <v>8</v>
+      </c>
+      <c r="O224" t="n">
+        <v>8</v>
+      </c>
+      <c r="R224" t="n">
+        <v>0.08881193827836725</v>
+      </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO224" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP224" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR224" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS224" t="inlineStr"/>
+      <c r="AT224" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU224" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV224" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW224" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX224" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY224" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ224" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA224" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB224" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC224" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>D038</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Influenza</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>流行性感冒</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N225" t="n">
+        <v>125</v>
+      </c>
+      <c r="O225" t="n">
+        <v>125</v>
+      </c>
+      <c r="R225" t="n">
+        <v>1.387686535599488</v>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO225" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP225" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR225" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS225" t="inlineStr"/>
+      <c r="AT225" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU225" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV225" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW225" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX225" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY225" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ225" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA225" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB225" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC225" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N226" t="n">
+        <v>1392</v>
+      </c>
+      <c r="O226" t="n">
+        <v>1392</v>
+      </c>
+      <c r="R226" t="n">
+        <v>15.4532772604359</v>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO226" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP226" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR226" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS226" t="inlineStr"/>
+      <c r="AT226" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU226" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV226" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW226" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX226" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY226" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ226" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA226" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB226" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC226" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N227" t="n">
+        <v>27</v>
+      </c>
+      <c r="O227" t="n">
+        <v>27</v>
+      </c>
+      <c r="R227" t="n">
+        <v>0.2997402916894895</v>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO227" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP227" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR227" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS227" t="inlineStr"/>
+      <c r="AT227" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU227" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV227" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW227" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX227" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY227" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ227" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA227" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB227" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC227" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N228" t="n">
+        <v>555</v>
+      </c>
+      <c r="O228" t="n">
+        <v>555</v>
+      </c>
+      <c r="R228" t="n">
+        <v>6.161328218061729</v>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO228" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP228" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR228" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS228" t="inlineStr"/>
+      <c r="AT228" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU228" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV228" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW228" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX228" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY228" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ228" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA228" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB228" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC228" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N229" t="n">
+        <v>261</v>
+      </c>
+      <c r="O229" t="n">
+        <v>261</v>
+      </c>
+      <c r="R229" t="n">
+        <v>2.897489486331732</v>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO229" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP229" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR229" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS229" t="inlineStr"/>
+      <c r="AT229" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU229" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV229" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW229" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX229" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY229" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ229" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA229" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB229" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC229" t="inlineStr">
         <is>
           <t>rest_api</t>
         </is>
@@ -33195,7 +34355,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
@@ -33278,7 +34438,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10">
@@ -33288,7 +34448,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>220</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11">
@@ -33340,7 +34500,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>54706</v>
+        <v>57231</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-18 00:06:26 UTC
</commit_message>
<xml_diff>
--- a/countries/ch/2026-2029.xlsx
+++ b/countries/ch/2026-2029.xlsx
@@ -14354,13 +14354,13 @@
         </is>
       </c>
       <c r="N94" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="O94" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="R94" t="n">
-        <v>2.897489486331732</v>
+        <v>2.886387994046936</v>
       </c>
       <c r="S94" t="inlineStr">
         <is>
@@ -19973,13 +19973,13 @@
         </is>
       </c>
       <c r="N132" t="n">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="O132" t="n">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="R132" t="n">
-        <v>4.351784975639996</v>
+        <v>4.3406834833552</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
@@ -25296,13 +25296,13 @@
         </is>
       </c>
       <c r="N168" t="n">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="O168" t="n">
-        <v>873</v>
+        <v>868</v>
       </c>
       <c r="R168" t="n">
-        <v>9.691602764626827</v>
+        <v>9.636095303202847</v>
       </c>
       <c r="S168" t="inlineStr">
         <is>
@@ -26414,13 +26414,13 @@
         </is>
       </c>
       <c r="N175" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="O175" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="R175" t="n">
-        <v>0.7437999830813258</v>
+        <v>0.721596998511734</v>
       </c>
       <c r="S175" t="inlineStr">
         <is>
@@ -29894,13 +29894,13 @@
         </is>
       </c>
       <c r="N199" t="n">
-        <v>2183</v>
+        <v>2173</v>
       </c>
       <c r="O199" t="n">
-        <v>2183</v>
+        <v>2173</v>
       </c>
       <c r="R199" t="n">
-        <v>24.23455765770947</v>
+        <v>24.12354273486151</v>
       </c>
       <c r="S199" t="inlineStr">
         <is>
@@ -30474,13 +30474,13 @@
         </is>
       </c>
       <c r="N203" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O203" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R203" t="n">
-        <v>0.2331313379807141</v>
+        <v>0.2442328302655099</v>
       </c>
       <c r="S203" t="inlineStr">
         <is>
@@ -30619,13 +30619,13 @@
         </is>
       </c>
       <c r="N204" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="O204" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="R204" t="n">
-        <v>1.365483551029897</v>
+        <v>1.398788027884284</v>
       </c>
       <c r="S204" t="inlineStr">
         <is>
@@ -32359,13 +32359,13 @@
         </is>
       </c>
       <c r="N216" t="n">
-        <v>1746</v>
+        <v>1737</v>
       </c>
       <c r="O216" t="n">
-        <v>1746</v>
+        <v>1737</v>
       </c>
       <c r="R216" t="n">
-        <v>19.38320552925365</v>
+        <v>19.28329209869049</v>
       </c>
       <c r="S216" t="inlineStr">
         <is>
@@ -32939,13 +32939,13 @@
         </is>
       </c>
       <c r="N220" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="O220" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="R220" t="n">
-        <v>0.1998268611263263</v>
+        <v>0.2553343225503059</v>
       </c>
       <c r="S220" t="inlineStr">
         <is>
@@ -33084,13 +33084,13 @@
         </is>
       </c>
       <c r="N221" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="O221" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="R221" t="n">
-        <v>1.121250720764387</v>
+        <v>1.143453705333978</v>
       </c>
       <c r="S221" t="inlineStr">
         <is>
@@ -33664,13 +33664,13 @@
         </is>
       </c>
       <c r="N225" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="O225" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="R225" t="n">
-        <v>1.387686535599488</v>
+        <v>1.432092504738672</v>
       </c>
       <c r="S225" t="inlineStr">
         <is>
@@ -34070,17 +34070,17 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>D114</t>
+          <t>D109</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Salmonellosis</t>
+          <t>Lyme disease</t>
         </is>
       </c>
       <c r="J228" t="inlineStr">
         <is>
-          <t>沙门氏菌病</t>
+          <t>莱姆病</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -34099,13 +34099,13 @@
         </is>
       </c>
       <c r="N228" t="n">
-        <v>555</v>
+        <v>1129</v>
       </c>
       <c r="O228" t="n">
-        <v>555</v>
+        <v>1129</v>
       </c>
       <c r="R228" t="n">
-        <v>6.161328218061729</v>
+        <v>12.53358478953458</v>
       </c>
       <c r="S228" t="inlineStr">
         <is>
@@ -34215,17 +34215,17 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>D115</t>
+          <t>D114</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>Shiga toxin-producing Escherichia coli infection</t>
+          <t>Salmonellosis</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>产志贺毒素大肠杆菌感染</t>
+          <t>沙门氏菌病</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -34244,13 +34244,13 @@
         </is>
       </c>
       <c r="N229" t="n">
-        <v>261</v>
+        <v>555</v>
       </c>
       <c r="O229" t="n">
-        <v>261</v>
+        <v>555</v>
       </c>
       <c r="R229" t="n">
-        <v>2.897489486331732</v>
+        <v>6.161328218061729</v>
       </c>
       <c r="S229" t="inlineStr">
         <is>
@@ -34317,6 +34317,441 @@
         </is>
       </c>
       <c r="BC229" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N230" t="n">
+        <v>261</v>
+      </c>
+      <c r="O230" t="n">
+        <v>261</v>
+      </c>
+      <c r="R230" t="n">
+        <v>2.897489486331732</v>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO230" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP230" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR230" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS230" t="inlineStr"/>
+      <c r="AT230" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU230" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV230" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW230" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX230" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY230" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ230" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA230" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB230" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC230" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>D123</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Tularemia</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>土拉菌病</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>8</v>
+      </c>
+      <c r="O231" t="n">
+        <v>8</v>
+      </c>
+      <c r="R231" t="n">
+        <v>0.08881193827836725</v>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO231" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP231" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR231" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS231" t="inlineStr"/>
+      <c r="AT231" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU231" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV231" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW231" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX231" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY231" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ231" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA231" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB231" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC231" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>D205</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>Tick-borne encephalitis</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>蜱传脑炎</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N232" t="n">
+        <v>25</v>
+      </c>
+      <c r="O232" t="n">
+        <v>25</v>
+      </c>
+      <c r="R232" t="n">
+        <v>0.2775373071198977</v>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO232" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP232" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR232" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS232" t="inlineStr"/>
+      <c r="AT232" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU232" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV232" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW232" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX232" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY232" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ232" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA232" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB232" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC232" t="inlineStr">
         <is>
           <t>rest_api</t>
         </is>
@@ -34438,7 +34873,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="10">
@@ -34448,7 +34883,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11">
@@ -34500,7 +34935,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>57231</v>
+        <v>58380</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-21 07:33:50 UTC
</commit_message>
<xml_diff>
--- a/countries/ch/2026-2029.xlsx
+++ b/countries/ch/2026-2029.xlsx
@@ -768,11 +768,6 @@
       <c r="R2" t="n">
         <v>0.954728336492448</v>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA2" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -785,23 +780,13 @@
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="n">
         <v>0</v>
       </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV2" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -915,17 +900,15 @@
       <c r="O3" t="n">
         <v>405</v>
       </c>
+      <c r="P3" t="n">
+        <v>405</v>
+      </c>
       <c r="Q3" t="n">
         <v>0</v>
       </c>
       <c r="R3" t="n">
         <v>4.496104375342342</v>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA3" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -938,23 +921,13 @@
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr"/>
       <c r="AT3" t="n">
         <v>0</v>
       </c>
-      <c r="AU3" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV3" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -1068,17 +1041,15 @@
       <c r="O4" t="n">
         <v>2743</v>
       </c>
+      <c r="P4" t="n">
+        <v>2743</v>
+      </c>
       <c r="Q4" t="n">
         <v>0</v>
       </c>
       <c r="R4" t="n">
         <v>30.45139333719517</v>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA4" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -1091,23 +1062,13 @@
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr"/>
       <c r="AT4" t="n">
         <v>0</v>
       </c>
-      <c r="AU4" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV4" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -1221,17 +1182,15 @@
       <c r="O5" t="n">
         <v>298</v>
       </c>
+      <c r="P5" t="n">
+        <v>298</v>
+      </c>
       <c r="Q5" t="n">
         <v>0</v>
       </c>
       <c r="R5" t="n">
         <v>3.30824470086918</v>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA5" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -1244,23 +1203,13 @@
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr"/>
       <c r="AT5" t="n">
         <v>0</v>
       </c>
-      <c r="AU5" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV5" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -1374,17 +1323,15 @@
       <c r="O6" t="n">
         <v>2287</v>
       </c>
+      <c r="P6" t="n">
+        <v>2287</v>
+      </c>
       <c r="Q6" t="n">
         <v>0</v>
       </c>
       <c r="R6" t="n">
         <v>25.38911285532824</v>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA6" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -1397,23 +1344,13 @@
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="n">
         <v>0</v>
       </c>
-      <c r="AU6" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV6" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -1527,17 +1464,15 @@
       <c r="O7" t="n">
         <v>248</v>
       </c>
+      <c r="P7" t="n">
+        <v>248</v>
+      </c>
       <c r="Q7" t="n">
         <v>0</v>
       </c>
       <c r="R7" t="n">
         <v>2.753170086629385</v>
       </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA7" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -1550,23 +1485,13 @@
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="n">
         <v>0</v>
       </c>
-      <c r="AU7" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV7" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -1680,17 +1605,15 @@
       <c r="O8" t="n">
         <v>1796</v>
       </c>
+      <c r="P8" t="n">
+        <v>1796</v>
+      </c>
       <c r="Q8" t="n">
         <v>0</v>
       </c>
       <c r="R8" t="n">
         <v>19.93828014349345</v>
       </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA8" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -1703,23 +1626,13 @@
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="n">
         <v>0</v>
       </c>
-      <c r="AU8" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV8" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -1833,17 +1746,15 @@
       <c r="O9" t="n">
         <v>240</v>
       </c>
+      <c r="P9" t="n">
+        <v>240</v>
+      </c>
       <c r="Q9" t="n">
         <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>2.664358148351018</v>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA9" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -1856,23 +1767,13 @@
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="n">
         <v>0</v>
       </c>
-      <c r="AU9" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV9" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -1986,17 +1887,15 @@
       <c r="O10" t="n">
         <v>1688</v>
       </c>
+      <c r="P10" t="n">
+        <v>1688</v>
+      </c>
       <c r="Q10" t="n">
         <v>0</v>
       </c>
       <c r="R10" t="n">
         <v>18.73931897673549</v>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA10" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -2009,23 +1908,13 @@
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="n">
         <v>0</v>
       </c>
-      <c r="AU10" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV10" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -2142,11 +2031,6 @@
       <c r="R11" t="n">
         <v>1.454295489308264</v>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA11" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -2159,23 +2043,13 @@
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR11" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="n">
         <v>0</v>
       </c>
-      <c r="AU11" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV11" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -2289,17 +2163,15 @@
       <c r="O12" t="n">
         <v>195</v>
       </c>
+      <c r="P12" t="n">
+        <v>195</v>
+      </c>
       <c r="Q12" t="n">
         <v>0</v>
       </c>
       <c r="R12" t="n">
         <v>2.164790995535202</v>
       </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA12" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -2312,23 +2184,13 @@
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR12" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="n">
         <v>0</v>
       </c>
-      <c r="AU12" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV12" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -2442,17 +2304,15 @@
       <c r="O13" t="n">
         <v>1232</v>
       </c>
+      <c r="P13" t="n">
+        <v>1232</v>
+      </c>
       <c r="Q13" t="n">
         <v>0</v>
       </c>
       <c r="R13" t="n">
         <v>13.67703849486856</v>
       </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA13" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -2465,23 +2325,13 @@
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR13" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="n">
         <v>0</v>
       </c>
-      <c r="AU13" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV13" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -2595,17 +2445,15 @@
       <c r="O14" t="n">
         <v>170</v>
       </c>
+      <c r="P14" t="n">
+        <v>170</v>
+      </c>
       <c r="Q14" t="n">
         <v>0</v>
       </c>
       <c r="R14" t="n">
         <v>1.887253688415304</v>
       </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA14" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -2618,23 +2466,13 @@
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="n">
         <v>0</v>
       </c>
-      <c r="AU14" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV14" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -2748,17 +2586,15 @@
       <c r="O15" t="n">
         <v>742</v>
       </c>
+      <c r="P15" t="n">
+        <v>742</v>
+      </c>
       <c r="Q15" t="n">
         <v>0</v>
       </c>
       <c r="R15" t="n">
         <v>8.237307275318562</v>
       </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA15" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -2771,23 +2607,13 @@
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="n">
         <v>0</v>
       </c>
-      <c r="AU15" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV15" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -2901,17 +2727,15 @@
       <c r="O16" t="n">
         <v>117</v>
       </c>
+      <c r="P16" t="n">
+        <v>117</v>
+      </c>
       <c r="Q16" t="n">
         <v>0</v>
       </c>
       <c r="R16" t="n">
         <v>1.298874597321121</v>
       </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA16" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -2924,23 +2748,13 @@
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr"/>
       <c r="AT16" t="n">
         <v>0</v>
       </c>
-      <c r="AU16" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV16" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -3054,17 +2868,15 @@
       <c r="O17" t="n">
         <v>386</v>
       </c>
+      <c r="P17" t="n">
+        <v>386</v>
+      </c>
       <c r="Q17" t="n">
         <v>0</v>
       </c>
       <c r="R17" t="n">
         <v>4.285176021931219</v>
       </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA17" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -3077,23 +2889,13 @@
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR17" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr"/>
       <c r="AT17" t="n">
         <v>0</v>
       </c>
-      <c r="AU17" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV17" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -3207,17 +3009,15 @@
       <c r="O18" t="n">
         <v>67</v>
       </c>
+      <c r="P18" t="n">
+        <v>67</v>
+      </c>
       <c r="Q18" t="n">
         <v>0</v>
       </c>
       <c r="R18" t="n">
         <v>0.7437999830813258</v>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA18" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -3230,23 +3030,13 @@
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR18" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr"/>
       <c r="AT18" t="n">
         <v>0</v>
       </c>
-      <c r="AU18" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV18" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -3360,17 +3150,15 @@
       <c r="O19" t="n">
         <v>238</v>
       </c>
+      <c r="P19" t="n">
+        <v>238</v>
+      </c>
       <c r="Q19" t="n">
         <v>0</v>
       </c>
       <c r="R19" t="n">
         <v>2.642155163781426</v>
       </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA19" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -3383,23 +3171,13 @@
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR19" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS19" t="inlineStr"/>
       <c r="AT19" t="n">
         <v>0</v>
       </c>
-      <c r="AU19" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV19" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -3516,11 +3294,6 @@
       <c r="R20" t="n">
         <v>2.908590978616528</v>
       </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA20" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -3533,23 +3306,13 @@
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR20" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS20" t="inlineStr"/>
       <c r="AT20" t="n">
         <v>0</v>
       </c>
-      <c r="AU20" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV20" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -3663,17 +3426,15 @@
       <c r="O21" t="n">
         <v>68</v>
       </c>
+      <c r="P21" t="n">
+        <v>68</v>
+      </c>
       <c r="Q21" t="n">
         <v>0</v>
       </c>
       <c r="R21" t="n">
         <v>0.7549014753661216</v>
       </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA21" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -3686,23 +3447,13 @@
       </c>
       <c r="AP21" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR21" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS21" t="inlineStr"/>
       <c r="AT21" t="n">
         <v>0</v>
       </c>
-      <c r="AU21" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV21" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -3816,17 +3567,15 @@
       <c r="O22" t="n">
         <v>130</v>
       </c>
+      <c r="P22" t="n">
+        <v>130</v>
+      </c>
       <c r="Q22" t="n">
         <v>0</v>
       </c>
       <c r="R22" t="n">
         <v>1.443193997023468</v>
       </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA22" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -3839,23 +3588,13 @@
       </c>
       <c r="AP22" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR22" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS22" t="inlineStr"/>
       <c r="AT22" t="n">
         <v>0</v>
       </c>
-      <c r="AU22" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV22" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -3969,14 +3708,12 @@
       <c r="O23" t="n">
         <v>44</v>
       </c>
+      <c r="P23" t="n">
+        <v>44</v>
+      </c>
       <c r="R23" t="n">
         <v>0.4884656605310199</v>
       </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA23" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -3989,23 +3726,13 @@
       </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR23" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS23" t="inlineStr"/>
       <c r="AT23" t="n">
         <v>0</v>
       </c>
-      <c r="AU23" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV23" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -4119,14 +3846,12 @@
       <c r="O24" t="n">
         <v>103</v>
       </c>
+      <c r="P24" t="n">
+        <v>103</v>
+      </c>
       <c r="R24" t="n">
         <v>1.143453705333978</v>
       </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA24" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -4139,23 +3864,13 @@
       </c>
       <c r="AP24" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR24" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS24" t="inlineStr"/>
       <c r="AT24" t="n">
         <v>0</v>
       </c>
-      <c r="AU24" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV24" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -4269,14 +3984,12 @@
       <c r="O25" t="n">
         <v>59</v>
       </c>
+      <c r="P25" t="n">
+        <v>59</v>
+      </c>
       <c r="R25" t="n">
         <v>0.6549880448029585</v>
       </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA25" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -4289,23 +4002,13 @@
       </c>
       <c r="AP25" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR25" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS25" t="inlineStr"/>
       <c r="AT25" t="n">
         <v>0</v>
       </c>
-      <c r="AU25" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV25" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -4419,14 +4122,12 @@
       <c r="O26" t="n">
         <v>67</v>
       </c>
+      <c r="P26" t="n">
+        <v>67</v>
+      </c>
       <c r="R26" t="n">
         <v>0.7437999830813258</v>
       </c>
-      <c r="S26" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA26" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -4439,23 +4140,13 @@
       </c>
       <c r="AP26" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR26" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS26" t="inlineStr"/>
       <c r="AT26" t="n">
         <v>0</v>
       </c>
-      <c r="AU26" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV26" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -4569,14 +4260,12 @@
       <c r="O27" t="n">
         <v>36</v>
       </c>
+      <c r="P27" t="n">
+        <v>36</v>
+      </c>
       <c r="R27" t="n">
         <v>0.3996537222526526</v>
       </c>
-      <c r="S27" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA27" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -4589,23 +4278,13 @@
       </c>
       <c r="AP27" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR27" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS27" t="inlineStr"/>
       <c r="AT27" t="n">
         <v>0</v>
       </c>
-      <c r="AU27" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV27" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -4719,14 +4398,12 @@
       <c r="O28" t="n">
         <v>50</v>
       </c>
+      <c r="P28" t="n">
+        <v>50</v>
+      </c>
       <c r="R28" t="n">
         <v>0.5550746142397954</v>
       </c>
-      <c r="S28" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA28" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -4739,23 +4416,13 @@
       </c>
       <c r="AP28" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR28" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS28" t="inlineStr"/>
       <c r="AT28" t="n">
         <v>0</v>
       </c>
-      <c r="AU28" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV28" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -4869,14 +4536,12 @@
       <c r="O29" t="n">
         <v>49</v>
       </c>
+      <c r="P29" t="n">
+        <v>49</v>
+      </c>
       <c r="R29" t="n">
         <v>0.5439731219549995</v>
       </c>
-      <c r="S29" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA29" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -4889,23 +4554,13 @@
       </c>
       <c r="AP29" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR29" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS29" t="inlineStr"/>
       <c r="AT29" t="n">
         <v>0</v>
       </c>
-      <c r="AU29" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV29" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -5019,14 +4674,12 @@
       <c r="O30" t="n">
         <v>52</v>
       </c>
+      <c r="P30" t="n">
+        <v>52</v>
+      </c>
       <c r="R30" t="n">
         <v>0.5772775988093871</v>
       </c>
-      <c r="S30" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA30" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -5039,23 +4692,13 @@
       </c>
       <c r="AP30" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR30" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS30" t="inlineStr"/>
       <c r="AT30" t="n">
         <v>0</v>
       </c>
-      <c r="AU30" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV30" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -5172,11 +4815,6 @@
       <c r="R31" t="n">
         <v>4.373987960209587</v>
       </c>
-      <c r="S31" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA31" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -5189,23 +4827,13 @@
       </c>
       <c r="AP31" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR31" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS31" t="inlineStr"/>
       <c r="AT31" t="n">
         <v>0</v>
       </c>
-      <c r="AU31" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV31" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -5319,14 +4947,12 @@
       <c r="O32" t="n">
         <v>27</v>
       </c>
+      <c r="P32" t="n">
+        <v>27</v>
+      </c>
       <c r="R32" t="n">
         <v>0.2997402916894895</v>
       </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA32" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -5339,23 +4965,13 @@
       </c>
       <c r="AP32" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR32" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS32" t="inlineStr"/>
       <c r="AT32" t="n">
         <v>0</v>
       </c>
-      <c r="AU32" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV32" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -5469,14 +5085,12 @@
       <c r="O33" t="n">
         <v>27</v>
       </c>
+      <c r="P33" t="n">
+        <v>27</v>
+      </c>
       <c r="R33" t="n">
         <v>0.2997402916894895</v>
       </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA33" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -5489,23 +5103,13 @@
       </c>
       <c r="AP33" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR33" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS33" t="inlineStr"/>
       <c r="AT33" t="n">
         <v>0</v>
       </c>
-      <c r="AU33" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV33" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -5619,14 +5223,12 @@
       <c r="O34" t="n">
         <v>25</v>
       </c>
+      <c r="P34" t="n">
+        <v>25</v>
+      </c>
       <c r="R34" t="n">
         <v>0.2775373071198977</v>
       </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA34" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -5639,23 +5241,13 @@
       </c>
       <c r="AP34" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR34" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS34" t="inlineStr"/>
       <c r="AT34" t="n">
         <v>0</v>
       </c>
-      <c r="AU34" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV34" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -5769,14 +5361,12 @@
       <c r="O35" t="n">
         <v>22</v>
       </c>
+      <c r="P35" t="n">
+        <v>22</v>
+      </c>
       <c r="R35" t="n">
         <v>0.2442328302655099</v>
       </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA35" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -5789,23 +5379,13 @@
       </c>
       <c r="AP35" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR35" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS35" t="inlineStr"/>
       <c r="AT35" t="n">
         <v>0</v>
       </c>
-      <c r="AU35" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV35" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -5919,14 +5499,12 @@
       <c r="O36" t="n">
         <v>9</v>
       </c>
+      <c r="P36" t="n">
+        <v>9</v>
+      </c>
       <c r="R36" t="n">
         <v>0.09991343056316315</v>
       </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA36" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -5939,23 +5517,13 @@
       </c>
       <c r="AP36" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR36" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS36" t="inlineStr"/>
       <c r="AT36" t="n">
         <v>0</v>
       </c>
-      <c r="AU36" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV36" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -6069,14 +5637,12 @@
       <c r="O37" t="n">
         <v>14</v>
       </c>
+      <c r="P37" t="n">
+        <v>14</v>
+      </c>
       <c r="R37" t="n">
         <v>0.1554208919871427</v>
       </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA37" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -6089,23 +5655,13 @@
       </c>
       <c r="AP37" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR37" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS37" t="inlineStr"/>
       <c r="AT37" t="n">
         <v>0</v>
       </c>
-      <c r="AU37" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV37" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -6219,14 +5775,12 @@
       <c r="O38" t="n">
         <v>11</v>
       </c>
+      <c r="P38" t="n">
+        <v>11</v>
+      </c>
       <c r="R38" t="n">
         <v>0.122116415132755</v>
       </c>
-      <c r="S38" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA38" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -6239,23 +5793,13 @@
       </c>
       <c r="AP38" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR38" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS38" t="inlineStr"/>
       <c r="AT38" t="n">
         <v>0</v>
       </c>
-      <c r="AU38" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV38" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -6369,14 +5913,12 @@
       <c r="O39" t="n">
         <v>8</v>
       </c>
+      <c r="P39" t="n">
+        <v>8</v>
+      </c>
       <c r="R39" t="n">
         <v>0.08881193827836725</v>
       </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA39" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -6389,23 +5931,13 @@
       </c>
       <c r="AP39" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR39" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS39" t="inlineStr"/>
       <c r="AT39" t="n">
         <v>0</v>
       </c>
-      <c r="AU39" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV39" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -6522,11 +6054,6 @@
       <c r="R40" t="n">
         <v>9.724907241481215</v>
       </c>
-      <c r="S40" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA40" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -6539,23 +6066,13 @@
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR40" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS40" t="inlineStr"/>
       <c r="AT40" t="n">
         <v>0</v>
       </c>
-      <c r="AU40" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV40" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -6669,14 +6186,12 @@
       <c r="O41" t="n">
         <v>14</v>
       </c>
+      <c r="P41" t="n">
+        <v>14</v>
+      </c>
       <c r="R41" t="n">
         <v>0.1554208919871427</v>
       </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA41" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -6689,23 +6204,13 @@
       </c>
       <c r="AP41" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR41" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS41" t="inlineStr"/>
       <c r="AT41" t="n">
         <v>0</v>
       </c>
-      <c r="AU41" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV41" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -6819,14 +6324,12 @@
       <c r="O42" t="n">
         <v>11</v>
       </c>
+      <c r="P42" t="n">
+        <v>11</v>
+      </c>
       <c r="R42" t="n">
         <v>0.122116415132755</v>
       </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA42" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -6839,23 +6342,13 @@
       </c>
       <c r="AP42" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR42" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS42" t="inlineStr"/>
       <c r="AT42" t="n">
         <v>0</v>
       </c>
-      <c r="AU42" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV42" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -6969,14 +6462,12 @@
       <c r="O43" t="n">
         <v>12</v>
       </c>
+      <c r="P43" t="n">
+        <v>12</v>
+      </c>
       <c r="R43" t="n">
         <v>0.1332179074175509</v>
       </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA43" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -6989,23 +6480,13 @@
       </c>
       <c r="AP43" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR43" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS43" t="inlineStr"/>
       <c r="AT43" t="n">
         <v>0</v>
       </c>
-      <c r="AU43" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV43" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -7119,14 +6600,12 @@
       <c r="O44" t="n">
         <v>10</v>
       </c>
+      <c r="P44" t="n">
+        <v>10</v>
+      </c>
       <c r="R44" t="n">
         <v>0.1110149228479591</v>
       </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA44" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -7139,23 +6618,13 @@
       </c>
       <c r="AP44" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR44" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS44" t="inlineStr"/>
       <c r="AT44" t="n">
         <v>0</v>
       </c>
-      <c r="AU44" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV44" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -7269,14 +6738,12 @@
       <c r="O45" t="n">
         <v>17</v>
       </c>
+      <c r="P45" t="n">
+        <v>17</v>
+      </c>
       <c r="R45" t="n">
         <v>0.1887253688415304</v>
       </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA45" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -7289,23 +6756,13 @@
       </c>
       <c r="AP45" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR45" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS45" t="inlineStr"/>
       <c r="AT45" t="n">
         <v>0</v>
       </c>
-      <c r="AU45" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV45" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -7419,14 +6876,12 @@
       <c r="O46" t="n">
         <v>11</v>
       </c>
+      <c r="P46" t="n">
+        <v>11</v>
+      </c>
       <c r="R46" t="n">
         <v>0.122116415132755</v>
       </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA46" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -7439,23 +6894,13 @@
       </c>
       <c r="AP46" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR46" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS46" t="inlineStr"/>
       <c r="AT46" t="n">
         <v>0</v>
       </c>
-      <c r="AU46" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV46" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -7569,14 +7014,12 @@
       <c r="O47" t="n">
         <v>7</v>
       </c>
+      <c r="P47" t="n">
+        <v>7</v>
+      </c>
       <c r="R47" t="n">
         <v>0.07771044599357135</v>
       </c>
-      <c r="S47" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA47" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -7589,23 +7032,13 @@
       </c>
       <c r="AP47" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR47" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS47" t="inlineStr"/>
       <c r="AT47" t="n">
         <v>0</v>
       </c>
-      <c r="AU47" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV47" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -7719,14 +7152,12 @@
       <c r="O48" t="n">
         <v>7</v>
       </c>
+      <c r="P48" t="n">
+        <v>7</v>
+      </c>
       <c r="R48" t="n">
         <v>0.07771044599357135</v>
       </c>
-      <c r="S48" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA48" t="inlineStr">
         <is>
           <t>weekly</t>
@@ -7739,23 +7170,13 @@
       </c>
       <c r="AP48" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR48" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS48" t="inlineStr"/>
       <c r="AT48" t="n">
         <v>0</v>
       </c>
-      <c r="AU48" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV48" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -7872,11 +7293,6 @@
       <c r="R49" t="n">
         <v>24.30116661141824</v>
       </c>
-      <c r="S49" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA49" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -7889,23 +7305,13 @@
       </c>
       <c r="AP49" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR49" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS49" t="inlineStr"/>
       <c r="AT49" t="n">
         <v>0</v>
       </c>
-      <c r="AU49" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV49" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -8022,11 +7428,6 @@
       <c r="R50" t="n">
         <v>19.43871299067763</v>
       </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA50" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -8039,23 +7440,13 @@
       </c>
       <c r="AP50" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR50" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS50" t="inlineStr"/>
       <c r="AT50" t="n">
         <v>0</v>
       </c>
-      <c r="AU50" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
-      </c>
       <c r="AV50" t="inlineStr">
         <is>
           <t>foph_idd</t>
@@ -8172,11 +7563,6 @@
       <c r="R51" t="n">
         <v>12.63349822009774</v>
       </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
       <c r="AA51" t="inlineStr">
         <is>
           <t>monthly</t>
@@ -8189,22 +7575,12 @@
       </c>
       <c r="AP51" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR51" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
+          <t>published_series</t>
         </is>
       </c>
       <c r="AS51" t="inlineStr"/>
       <c r="AT51" t="n">
         <v>0</v>
-      </c>
-      <c r="AU51" t="inlineStr">
-        <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
-        </is>
       </c>
       <c r="AV51" t="inlineStr">
         <is>

</xml_diff>